<commit_message>
Split the README into docs/ pages; add "How to add new things"
- README.md is now a one-page overview: what it is, a quick start, a table
  of the docs, and what's in the repository.
- docs/: setup and everyday use, collecting the data (order of work and
  measuring protocol), how to add new things (a recipe per kind of thing),
  spreadsheet reference, the checks and the report, rearranging in
  Inkscape, decommissioning, the lab directory, for developers.
- Cross-references are links now; the example README, the shapes template
  and the workbooks' help sheet point at the right pages.
- Fixed a stale line: stacks no longer move as one in the flat layout.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lab-data.xlsx
+++ b/lab-data.xlsx
@@ -1375,7 +1375,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Photos and SOPs aren't listed here: they're linked by file name (see README.md).</t>
+          <t>Photos and SOPs aren't listed here: they're linked by file name (see docs/adding-things.md).</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Full guide: README.md in this folder. Worked example: example/lab-data.xlsx.</t>
+          <t>Full guide: README.md and the docs folder. Worked example: example/lab-data.xlsx.</t>
         </is>
       </c>
     </row>

</xml_diff>